<commit_message>
modify age range for Policia and SNMV
</commit_message>
<xml_diff>
--- a/data/Sistema_de_Notificacion_de_Muertes_Violentas/svmvIncidentes.xlsx
+++ b/data/Sistema_de_Notificacion_de_Muertes_Violentas/svmvIncidentes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Sistema_de_Notificacion_de_Muertes_Violentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9664275B-DA21-400F-A954-CC1141F75C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CAD21E1-1797-4B51-8C5A-25351B66BCDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{9CFC54A2-FB65-C045-ACC9-D5EBAFBDCE35}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{9CFC54A2-FB65-C045-ACC9-D5EBAFBDCE35}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -101,7 +101,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -109,17 +109,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -441,7 +459,7 @@
     <col min="1" max="1" width="53.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -479,7 +497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -510,15 +528,15 @@
       <c r="J2" s="1">
         <v>33</v>
       </c>
-      <c r="K2" s="1">
-        <v>19</v>
+      <c r="K2" s="3">
+        <v>24</v>
       </c>
       <c r="L2" s="1">
         <f t="shared" ref="L2:L8" si="0">SUM(B2:K2)</f>
-        <v>362</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -549,15 +567,15 @@
       <c r="J3" s="1">
         <v>41</v>
       </c>
-      <c r="K3" s="1">
-        <v>21</v>
+      <c r="K3" s="3">
+        <v>24</v>
       </c>
       <c r="L3" s="1">
         <f t="shared" si="0"/>
-        <v>284</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -588,7 +606,7 @@
       <c r="J4" s="1">
         <v>0</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="3">
         <v>0</v>
       </c>
       <c r="L4" s="1">
@@ -596,7 +614,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -627,7 +645,7 @@
       <c r="J5" s="1">
         <v>0</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="3">
         <v>0</v>
       </c>
       <c r="L5" s="1">
@@ -635,7 +653,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -666,7 +684,7 @@
       <c r="J6" s="1">
         <v>0</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="3">
         <v>0</v>
       </c>
       <c r="L6" s="1">
@@ -674,7 +692,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -705,15 +723,15 @@
       <c r="J7" s="1">
         <v>4</v>
       </c>
-      <c r="K7" s="1">
-        <v>0</v>
+      <c r="K7" s="3">
+        <v>1</v>
       </c>
       <c r="L7" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -744,7 +762,7 @@
       <c r="J8" s="1">
         <v>0</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="3">
         <v>0</v>
       </c>
       <c r="L8" s="1">
@@ -752,7 +770,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -783,7 +801,7 @@
       <c r="J9" s="1">
         <v>13</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="3">
         <v>2</v>
       </c>
       <c r="L9" s="1">
@@ -791,7 +809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -820,14 +838,14 @@
         <v>96</v>
       </c>
       <c r="J10" s="2">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="K10" s="2">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="L10" s="1">
         <f>SUM(B10:K10)</f>
-        <v>834</v>
+        <v>845</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -859,14 +877,14 @@
         <v>100</v>
       </c>
       <c r="J11" s="1">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K11" s="1">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="L11" s="1">
         <f>SUM(B11:K11)</f>
-        <v>849</v>
+        <v>857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>